<commit_message>
Correzione nomi AGV e tempo trasp lam = 1/6
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_AGV/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_AGV/FOLDER/EXCEL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_AGV\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C0D36F-F949-4D0B-90A3-5B6EFBF9CB7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5953972F-DC98-416C-8315-3A3112F9C065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -442,11 +442,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -738,26 +738,26 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
+      <c r="A3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
     </row>
     <row r="4" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -2438,26 +2438,26 @@
       </c>
     </row>
     <row r="34" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="9"/>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
-      <c r="M34" s="9"/>
-      <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="9"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="10"/>
     </row>
     <row r="35" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -4138,26 +4138,26 @@
       </c>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A65" s="9" t="s">
+      <c r="A65" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="9"/>
-      <c r="J65" s="9"/>
-      <c r="K65" s="9"/>
-      <c r="L65" s="9"/>
-      <c r="M65" s="9"/>
-      <c r="N65" s="9"/>
-      <c r="O65" s="9"/>
-      <c r="P65" s="9"/>
-      <c r="Q65" s="9"/>
-      <c r="R65" s="9"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="10"/>
+      <c r="F65" s="10"/>
+      <c r="G65" s="10"/>
+      <c r="H65" s="10"/>
+      <c r="I65" s="10"/>
+      <c r="J65" s="10"/>
+      <c r="K65" s="10"/>
+      <c r="L65" s="10"/>
+      <c r="M65" s="10"/>
+      <c r="N65" s="10"/>
+      <c r="O65" s="10"/>
+      <c r="P65" s="10"/>
+      <c r="Q65" s="10"/>
+      <c r="R65" s="10"/>
     </row>
     <row r="66" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
@@ -5838,26 +5838,26 @@
       </c>
     </row>
     <row r="96" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A96" s="9" t="s">
+      <c r="A96" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9"/>
-      <c r="D96" s="9"/>
-      <c r="E96" s="9"/>
-      <c r="F96" s="9"/>
-      <c r="G96" s="9"/>
-      <c r="H96" s="9"/>
-      <c r="I96" s="9"/>
-      <c r="J96" s="9"/>
-      <c r="K96" s="9"/>
-      <c r="L96" s="9"/>
-      <c r="M96" s="9"/>
-      <c r="N96" s="9"/>
-      <c r="O96" s="9"/>
-      <c r="P96" s="9"/>
-      <c r="Q96" s="9"/>
-      <c r="R96" s="9"/>
+      <c r="B96" s="10"/>
+      <c r="C96" s="10"/>
+      <c r="D96" s="10"/>
+      <c r="E96" s="10"/>
+      <c r="F96" s="10"/>
+      <c r="G96" s="10"/>
+      <c r="H96" s="10"/>
+      <c r="I96" s="10"/>
+      <c r="J96" s="10"/>
+      <c r="K96" s="10"/>
+      <c r="L96" s="10"/>
+      <c r="M96" s="10"/>
+      <c r="N96" s="10"/>
+      <c r="O96" s="10"/>
+      <c r="P96" s="10"/>
+      <c r="Q96" s="10"/>
+      <c r="R96" s="10"/>
     </row>
     <row r="97" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
@@ -7538,38 +7538,38 @@
       </c>
     </row>
     <row r="127" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A127" s="9" t="s">
+      <c r="A127" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B127" s="9"/>
-      <c r="C127" s="9"/>
-      <c r="D127" s="9"/>
-      <c r="E127" s="9"/>
-      <c r="F127" s="9"/>
-      <c r="G127" s="9"/>
-      <c r="H127" s="9"/>
-      <c r="I127" s="9"/>
-      <c r="J127" s="9"/>
-      <c r="K127" s="9"/>
-      <c r="L127" s="9"/>
-      <c r="M127" s="9"/>
-      <c r="N127" s="9"/>
-      <c r="O127" s="9"/>
-      <c r="P127" s="9"/>
-      <c r="Q127" s="9"/>
-      <c r="R127" s="9"/>
-      <c r="S127" s="9"/>
-      <c r="T127" s="9"/>
-      <c r="U127" s="9"/>
-      <c r="V127" s="9"/>
-      <c r="W127" s="9"/>
-      <c r="X127" s="9"/>
-      <c r="Y127" s="9"/>
-      <c r="Z127" s="9"/>
-      <c r="AA127" s="9"/>
-      <c r="AB127" s="9"/>
-      <c r="AC127" s="9"/>
-      <c r="AD127" s="9"/>
+      <c r="B127" s="10"/>
+      <c r="C127" s="10"/>
+      <c r="D127" s="10"/>
+      <c r="E127" s="10"/>
+      <c r="F127" s="10"/>
+      <c r="G127" s="10"/>
+      <c r="H127" s="10"/>
+      <c r="I127" s="10"/>
+      <c r="J127" s="10"/>
+      <c r="K127" s="10"/>
+      <c r="L127" s="10"/>
+      <c r="M127" s="10"/>
+      <c r="N127" s="10"/>
+      <c r="O127" s="10"/>
+      <c r="P127" s="10"/>
+      <c r="Q127" s="10"/>
+      <c r="R127" s="10"/>
+      <c r="S127" s="10"/>
+      <c r="T127" s="10"/>
+      <c r="U127" s="10"/>
+      <c r="V127" s="10"/>
+      <c r="W127" s="10"/>
+      <c r="X127" s="10"/>
+      <c r="Y127" s="10"/>
+      <c r="Z127" s="10"/>
+      <c r="AA127" s="10"/>
+      <c r="AB127" s="10"/>
+      <c r="AC127" s="10"/>
+      <c r="AD127" s="10"/>
     </row>
     <row r="128" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A128" s="2"/>
@@ -7846,25 +7846,25 @@
       </c>
     </row>
     <row r="131" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A131" s="9" t="s">
+      <c r="A131" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B131" s="9"/>
-      <c r="C131" s="9"/>
-      <c r="D131" s="9"/>
-      <c r="E131" s="9"/>
-      <c r="F131" s="9"/>
-      <c r="G131" s="9"/>
-      <c r="H131" s="9"/>
-      <c r="I131" s="9"/>
-      <c r="J131" s="9"/>
-      <c r="K131" s="9"/>
-      <c r="L131" s="9"/>
-      <c r="M131" s="9"/>
-      <c r="N131" s="9"/>
-      <c r="O131" s="9"/>
-      <c r="P131" s="9"/>
-      <c r="Q131" s="9"/>
+      <c r="B131" s="10"/>
+      <c r="C131" s="10"/>
+      <c r="D131" s="10"/>
+      <c r="E131" s="10"/>
+      <c r="F131" s="10"/>
+      <c r="G131" s="10"/>
+      <c r="H131" s="10"/>
+      <c r="I131" s="10"/>
+      <c r="J131" s="10"/>
+      <c r="K131" s="10"/>
+      <c r="L131" s="10"/>
+      <c r="M131" s="10"/>
+      <c r="N131" s="10"/>
+      <c r="O131" s="10"/>
+      <c r="P131" s="10"/>
+      <c r="Q131" s="10"/>
     </row>
     <row r="132" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
@@ -8197,7 +8197,7 @@
         <v>0.125</v>
       </c>
       <c r="Q140" s="8">
-        <v>0.1111111111111111</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="141" spans="1:30" x14ac:dyDescent="0.3">
@@ -8389,6 +8389,5 @@
     <mergeCell ref="A127:AD127"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel e Matlab AGV
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_AGV/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_AGV/FOLDER/EXCEL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_AGV\FOLDER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_AGV\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5953972F-DC98-416C-8315-3A3112F9C065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4EF1FD-D35B-4766-8D3D-47E67184A167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5520" yWindow="3015" windowWidth="6330" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -443,10 +443,10 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -730,36 +730,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AD147"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-    </row>
-    <row r="4" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+    </row>
+    <row r="4" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -813,7 +813,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
@@ -869,7 +869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
@@ -925,7 +925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
@@ -981,7 +981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>22</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>23</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>24</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>26</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>27</v>
       </c>
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>28</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>29</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>30</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>31</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>32</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>33</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>34</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>35</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>36</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>37</v>
       </c>
@@ -1877,7 +1877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>38</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>39</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>40</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>41</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>42</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>43</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>44</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>45</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>46</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>47</v>
       </c>
@@ -2437,29 +2437,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
-      <c r="M34" s="10"/>
-      <c r="N34" s="10"/>
-      <c r="O34" s="10"/>
-      <c r="P34" s="10"/>
-      <c r="Q34" s="10"/>
-      <c r="R34" s="10"/>
-    </row>
-    <row r="35" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+    </row>
+    <row r="35" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="3" t="s">
         <v>2</v>
@@ -2513,7 +2513,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>19</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>20</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>21</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>22</v>
       </c>
@@ -2737,7 +2737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>23</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>24</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>25</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>26</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>27</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>28</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>29</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>30</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>31</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>32</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>33</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>34</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>35</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>36</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>37</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>38</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>39</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>40</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>41</v>
       </c>
@@ -3801,7 +3801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>42</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>43</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
         <v>44</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>45</v>
       </c>
@@ -4025,7 +4025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
         <v>46</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>47</v>
       </c>
@@ -4137,29 +4137,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A65" s="10" t="s">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A65" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="10"/>
-      <c r="G65" s="10"/>
-      <c r="H65" s="10"/>
-      <c r="I65" s="10"/>
-      <c r="J65" s="10"/>
-      <c r="K65" s="10"/>
-      <c r="L65" s="10"/>
-      <c r="M65" s="10"/>
-      <c r="N65" s="10"/>
-      <c r="O65" s="10"/>
-      <c r="P65" s="10"/>
-      <c r="Q65" s="10"/>
-      <c r="R65" s="10"/>
-    </row>
-    <row r="66" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
+      <c r="I65" s="9"/>
+      <c r="J65" s="9"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="9"/>
+      <c r="M65" s="9"/>
+      <c r="N65" s="9"/>
+      <c r="O65" s="9"/>
+      <c r="P65" s="9"/>
+      <c r="Q65" s="9"/>
+      <c r="R65" s="9"/>
+    </row>
+    <row r="66" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="3" t="s">
         <v>2</v>
@@ -4213,7 +4213,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>19</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>20</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>21</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>22</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>23</v>
       </c>
@@ -4493,7 +4493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>24</v>
       </c>
@@ -4549,7 +4549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>25</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>26</v>
       </c>
@@ -4661,7 +4661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>27</v>
       </c>
@@ -4717,7 +4717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>28</v>
       </c>
@@ -4773,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>29</v>
       </c>
@@ -4829,7 +4829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>30</v>
       </c>
@@ -4885,7 +4885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>31</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>32</v>
       </c>
@@ -4997,7 +4997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>33</v>
       </c>
@@ -5053,7 +5053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>34</v>
       </c>
@@ -5109,7 +5109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>35</v>
       </c>
@@ -5165,7 +5165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>36</v>
       </c>
@@ -5221,7 +5221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>37</v>
       </c>
@@ -5277,7 +5277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>38</v>
       </c>
@@ -5333,7 +5333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>39</v>
       </c>
@@ -5389,7 +5389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>40</v>
       </c>
@@ -5445,7 +5445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>41</v>
       </c>
@@ -5501,7 +5501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>42</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>43</v>
       </c>
@@ -5613,7 +5613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>44</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>45</v>
       </c>
@@ -5725,7 +5725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>46</v>
       </c>
@@ -5781,7 +5781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>47</v>
       </c>
@@ -5837,29 +5837,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A96" s="10" t="s">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A96" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B96" s="10"/>
-      <c r="C96" s="10"/>
-      <c r="D96" s="10"/>
-      <c r="E96" s="10"/>
-      <c r="F96" s="10"/>
-      <c r="G96" s="10"/>
-      <c r="H96" s="10"/>
-      <c r="I96" s="10"/>
-      <c r="J96" s="10"/>
-      <c r="K96" s="10"/>
-      <c r="L96" s="10"/>
-      <c r="M96" s="10"/>
-      <c r="N96" s="10"/>
-      <c r="O96" s="10"/>
-      <c r="P96" s="10"/>
-      <c r="Q96" s="10"/>
-      <c r="R96" s="10"/>
-    </row>
-    <row r="97" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B96" s="9"/>
+      <c r="C96" s="9"/>
+      <c r="D96" s="9"/>
+      <c r="E96" s="9"/>
+      <c r="F96" s="9"/>
+      <c r="G96" s="9"/>
+      <c r="H96" s="9"/>
+      <c r="I96" s="9"/>
+      <c r="J96" s="9"/>
+      <c r="K96" s="9"/>
+      <c r="L96" s="9"/>
+      <c r="M96" s="9"/>
+      <c r="N96" s="9"/>
+      <c r="O96" s="9"/>
+      <c r="P96" s="9"/>
+      <c r="Q96" s="9"/>
+      <c r="R96" s="9"/>
+    </row>
+    <row r="97" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="3" t="s">
         <v>2</v>
@@ -5913,7 +5913,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
         <v>19</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
         <v>20</v>
       </c>
@@ -6025,7 +6025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
         <v>21</v>
       </c>
@@ -6081,7 +6081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
         <v>22</v>
       </c>
@@ -6137,7 +6137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
         <v>23</v>
       </c>
@@ -6193,7 +6193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
         <v>24</v>
       </c>
@@ -6249,7 +6249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
         <v>25</v>
       </c>
@@ -6305,7 +6305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
         <v>26</v>
       </c>
@@ -6361,7 +6361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
         <v>27</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>28</v>
       </c>
@@ -6473,7 +6473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>29</v>
       </c>
@@ -6529,7 +6529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>30</v>
       </c>
@@ -6585,7 +6585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
         <v>31</v>
       </c>
@@ -6641,7 +6641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
         <v>32</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
         <v>33</v>
       </c>
@@ -6753,7 +6753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
         <v>34</v>
       </c>
@@ -6809,7 +6809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>35</v>
       </c>
@@ -6865,7 +6865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
         <v>36</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
         <v>37</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
         <v>38</v>
       </c>
@@ -7033,7 +7033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
         <v>39</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
         <v>40</v>
       </c>
@@ -7145,7 +7145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
         <v>41</v>
       </c>
@@ -7201,7 +7201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
         <v>42</v>
       </c>
@@ -7257,7 +7257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
         <v>43</v>
       </c>
@@ -7313,7 +7313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
         <v>44</v>
       </c>
@@ -7369,7 +7369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
         <v>45</v>
       </c>
@@ -7425,7 +7425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:30" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:30" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
         <v>46</v>
       </c>
@@ -7481,7 +7481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
         <v>47</v>
       </c>
@@ -7537,41 +7537,41 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A127" s="10" t="s">
+    <row r="127" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A127" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B127" s="10"/>
-      <c r="C127" s="10"/>
-      <c r="D127" s="10"/>
-      <c r="E127" s="10"/>
-      <c r="F127" s="10"/>
-      <c r="G127" s="10"/>
-      <c r="H127" s="10"/>
-      <c r="I127" s="10"/>
-      <c r="J127" s="10"/>
-      <c r="K127" s="10"/>
-      <c r="L127" s="10"/>
-      <c r="M127" s="10"/>
-      <c r="N127" s="10"/>
-      <c r="O127" s="10"/>
-      <c r="P127" s="10"/>
-      <c r="Q127" s="10"/>
-      <c r="R127" s="10"/>
-      <c r="S127" s="10"/>
-      <c r="T127" s="10"/>
-      <c r="U127" s="10"/>
-      <c r="V127" s="10"/>
-      <c r="W127" s="10"/>
-      <c r="X127" s="10"/>
-      <c r="Y127" s="10"/>
-      <c r="Z127" s="10"/>
-      <c r="AA127" s="10"/>
-      <c r="AB127" s="10"/>
-      <c r="AC127" s="10"/>
-      <c r="AD127" s="10"/>
-    </row>
-    <row r="128" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B127" s="9"/>
+      <c r="C127" s="9"/>
+      <c r="D127" s="9"/>
+      <c r="E127" s="9"/>
+      <c r="F127" s="9"/>
+      <c r="G127" s="9"/>
+      <c r="H127" s="9"/>
+      <c r="I127" s="9"/>
+      <c r="J127" s="9"/>
+      <c r="K127" s="9"/>
+      <c r="L127" s="9"/>
+      <c r="M127" s="9"/>
+      <c r="N127" s="9"/>
+      <c r="O127" s="9"/>
+      <c r="P127" s="9"/>
+      <c r="Q127" s="9"/>
+      <c r="R127" s="9"/>
+      <c r="S127" s="9"/>
+      <c r="T127" s="9"/>
+      <c r="U127" s="9"/>
+      <c r="V127" s="9"/>
+      <c r="W127" s="9"/>
+      <c r="X127" s="9"/>
+      <c r="Y127" s="9"/>
+      <c r="Z127" s="9"/>
+      <c r="AA127" s="9"/>
+      <c r="AB127" s="9"/>
+      <c r="AC127" s="9"/>
+      <c r="AD127" s="9"/>
+    </row>
+    <row r="128" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="3" t="s">
         <v>19</v>
@@ -7661,7 +7661,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="129" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
         <v>52</v>
       </c>
@@ -7753,7 +7753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
         <v>53</v>
       </c>
@@ -7845,28 +7845,28 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A131" s="10" t="s">
+    <row r="131" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A131" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B131" s="10"/>
-      <c r="C131" s="10"/>
-      <c r="D131" s="10"/>
-      <c r="E131" s="10"/>
-      <c r="F131" s="10"/>
-      <c r="G131" s="10"/>
-      <c r="H131" s="10"/>
-      <c r="I131" s="10"/>
-      <c r="J131" s="10"/>
-      <c r="K131" s="10"/>
-      <c r="L131" s="10"/>
-      <c r="M131" s="10"/>
-      <c r="N131" s="10"/>
-      <c r="O131" s="10"/>
-      <c r="P131" s="10"/>
-      <c r="Q131" s="10"/>
-    </row>
-    <row r="132" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B131" s="9"/>
+      <c r="C131" s="9"/>
+      <c r="D131" s="9"/>
+      <c r="E131" s="9"/>
+      <c r="F131" s="9"/>
+      <c r="G131" s="9"/>
+      <c r="H131" s="9"/>
+      <c r="I131" s="9"/>
+      <c r="J131" s="9"/>
+      <c r="K131" s="9"/>
+      <c r="L131" s="9"/>
+      <c r="M131" s="9"/>
+      <c r="N131" s="9"/>
+      <c r="O131" s="9"/>
+      <c r="P131" s="9"/>
+      <c r="Q131" s="9"/>
+    </row>
+    <row r="132" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>2</v>
       </c>
@@ -7919,7 +7919,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="133" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
         <v>55</v>
       </c>
@@ -7972,12 +7972,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="134" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="135" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:30" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>2</v>
       </c>
@@ -8030,7 +8030,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="136" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>55</v>
       </c>
@@ -8083,13 +8083,13 @@
         <v>55</v>
       </c>
     </row>
-    <row r="137" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>57</v>
       </c>
       <c r="J137" s="7"/>
     </row>
-    <row r="138" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>0</v>
       </c>
@@ -8142,12 +8142,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="140" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A140" s="8">
         <v>0.5</v>
       </c>
@@ -8200,12 +8200,12 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="141" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="142" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>0</v>
       </c>
@@ -8258,12 +8258,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="144" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>0</v>
       </c>
@@ -8316,12 +8316,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>0</v>
       </c>
@@ -8374,7 +8374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>62</v>
       </c>

</xml_diff>